<commit_message>
Sync data files - 2025-08-19 08:08:39 (       2 files updated)
</commit_message>
<xml_diff>
--- a/Data/Transactions/Sidra_transactions.xlsx
+++ b/Data/Transactions/Sidra_transactions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/levan/Documents/MegaValuationer/Data/Transactions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F383D5-2D3D-A944-A194-67E41746F968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B266E32-9236-974B-AAB2-8C9222C2390A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{A799E9DF-2EC2-BB4D-96E3-8DA9F4319B01}"/>
   </bookViews>
@@ -3360,9 +3360,6 @@
     <t>Community/Building</t>
   </si>
   <si>
-    <t>Sub Community / Building</t>
-  </si>
-  <si>
     <t>Beds</t>
   </si>
   <si>
@@ -3664,6 +3661,9 @@
   </si>
   <si>
     <t>DE Sidra 3-V-61</t>
+  </si>
+  <si>
+    <t>Sub Community/Building</t>
   </si>
 </sst>
 </file>
@@ -4078,34 +4078,34 @@
         <v>1105</v>
       </c>
       <c r="E1" t="s">
+        <v>1207</v>
+      </c>
+      <c r="F1" t="s">
         <v>1106</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>1107</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>1108</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>1109</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>1110</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>1111</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>1112</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>1113</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>1114</v>
-      </c>
-      <c r="N1" t="s">
-        <v>1115</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
@@ -4410,7 +4410,7 @@
         <v>7</v>
       </c>
       <c r="M8" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="N8" t="s">
         <v>9</v>
@@ -38686,7 +38686,7 @@
         <v>7</v>
       </c>
       <c r="M787" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="N787" t="s">
         <v>77</v>
@@ -38862,7 +38862,7 @@
         <v>7</v>
       </c>
       <c r="M791" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="N791" t="s">
         <v>77</v>
@@ -39170,7 +39170,7 @@
         <v>7</v>
       </c>
       <c r="M798" s="3" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="N798" t="s">
         <v>77</v>
@@ -40226,7 +40226,7 @@
         <v>7</v>
       </c>
       <c r="M822" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="N822" t="s">
         <v>9</v>
@@ -40358,7 +40358,7 @@
         <v>7</v>
       </c>
       <c r="M825" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="N825" t="s">
         <v>9</v>
@@ -41634,7 +41634,7 @@
         <v>7</v>
       </c>
       <c r="M854" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="N854" t="s">
         <v>77</v>
@@ -42954,7 +42954,7 @@
         <v>7</v>
       </c>
       <c r="M884" s="3" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="N884" t="s">
         <v>77</v>
@@ -44186,7 +44186,7 @@
         <v>7</v>
       </c>
       <c r="M912" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="N912" t="s">
         <v>77</v>
@@ -44494,7 +44494,7 @@
         <v>7</v>
       </c>
       <c r="M919" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="N919" t="s">
         <v>77</v>
@@ -45066,7 +45066,7 @@
         <v>7</v>
       </c>
       <c r="M932" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="N932" t="s">
         <v>9</v>
@@ -45682,7 +45682,7 @@
         <v>7</v>
       </c>
       <c r="M946" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="N946" t="s">
         <v>9</v>
@@ -45726,7 +45726,7 @@
         <v>7</v>
       </c>
       <c r="M947" s="3" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="N947" t="s">
         <v>77</v>
@@ -46254,7 +46254,7 @@
         <v>7</v>
       </c>
       <c r="M959" s="3" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="N959" t="s">
         <v>77</v>
@@ -46874,7 +46874,7 @@
         <v>7</v>
       </c>
       <c r="M973" s="3" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="N973" t="s">
         <v>77</v>
@@ -46962,7 +46962,7 @@
         <v>7</v>
       </c>
       <c r="M975" s="3" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="N975" t="s">
         <v>9</v>
@@ -47270,7 +47270,7 @@
         <v>7</v>
       </c>
       <c r="M982" s="3" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="N982" t="s">
         <v>77</v>
@@ -47490,7 +47490,7 @@
         <v>7</v>
       </c>
       <c r="M987" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="N987" t="s">
         <v>77</v>
@@ -47710,7 +47710,7 @@
         <v>7</v>
       </c>
       <c r="M992" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="N992" t="s">
         <v>77</v>
@@ -47754,7 +47754,7 @@
         <v>7</v>
       </c>
       <c r="M993" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="N993" t="s">
         <v>77</v>
@@ -48062,7 +48062,7 @@
         <v>7</v>
       </c>
       <c r="M1000" s="3" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="N1000" t="s">
         <v>77</v>
@@ -48194,7 +48194,7 @@
         <v>7</v>
       </c>
       <c r="M1003" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="N1003" t="s">
         <v>77</v>
@@ -49778,7 +49778,7 @@
         <v>7</v>
       </c>
       <c r="M1039" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="N1039" t="s">
         <v>77</v>
@@ -50086,7 +50086,7 @@
         <v>7</v>
       </c>
       <c r="M1046" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="N1046" t="s">
         <v>77</v>
@@ -50130,7 +50130,7 @@
         <v>7</v>
       </c>
       <c r="M1047" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="N1047" t="s">
         <v>77</v>
@@ -50262,7 +50262,7 @@
         <v>7</v>
       </c>
       <c r="M1050" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="N1050" t="s">
         <v>77</v>
@@ -51406,7 +51406,7 @@
         <v>7</v>
       </c>
       <c r="M1076" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="N1076" t="s">
         <v>77</v>
@@ -51670,7 +51670,7 @@
         <v>7</v>
       </c>
       <c r="M1082" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="N1082" t="s">
         <v>77</v>
@@ -51714,7 +51714,7 @@
         <v>7</v>
       </c>
       <c r="M1083" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="N1083" t="s">
         <v>77</v>
@@ -52110,7 +52110,7 @@
         <v>7</v>
       </c>
       <c r="M1092" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="N1092" t="s">
         <v>77</v>
@@ -52242,7 +52242,7 @@
         <v>7</v>
       </c>
       <c r="M1095" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="N1095" t="s">
         <v>77</v>
@@ -52286,7 +52286,7 @@
         <v>7</v>
       </c>
       <c r="M1096" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="N1096" t="s">
         <v>77</v>
@@ -52462,7 +52462,7 @@
         <v>7</v>
       </c>
       <c r="M1100" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="N1100" t="s">
         <v>77</v>
@@ -52682,7 +52682,7 @@
         <v>7</v>
       </c>
       <c r="M1105" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="N1105" t="s">
         <v>77</v>
@@ -53254,7 +53254,7 @@
         <v>7</v>
       </c>
       <c r="M1118" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="N1118" t="s">
         <v>77</v>
@@ -53342,7 +53342,7 @@
         <v>7</v>
       </c>
       <c r="M1120" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="N1120" t="s">
         <v>77</v>
@@ -53386,7 +53386,7 @@
         <v>7</v>
       </c>
       <c r="M1121" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="N1121" t="s">
         <v>77</v>
@@ -58666,7 +58666,7 @@
         <v>5</v>
       </c>
       <c r="M1241" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="N1241" t="s">
         <v>77</v>
@@ -60778,7 +60778,7 @@
         <v>7</v>
       </c>
       <c r="M1289" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="N1289" t="s">
         <v>77</v>
@@ -62582,7 +62582,7 @@
         <v>7</v>
       </c>
       <c r="M1330" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="N1330" t="s">
         <v>77</v>
@@ -62978,7 +62978,7 @@
         <v>7</v>
       </c>
       <c r="M1339" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="N1339" t="s">
         <v>77</v>
@@ -63286,7 +63286,7 @@
         <v>7</v>
       </c>
       <c r="M1346" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="N1346" t="s">
         <v>77</v>
@@ -63462,7 +63462,7 @@
         <v>7</v>
       </c>
       <c r="M1350" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="N1350" t="s">
         <v>77</v>
@@ -63638,7 +63638,7 @@
         <v>7</v>
       </c>
       <c r="M1354" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="N1354" t="s">
         <v>77</v>
@@ -63682,7 +63682,7 @@
         <v>7</v>
       </c>
       <c r="M1355" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="N1355" t="s">
         <v>77</v>
@@ -63814,7 +63814,7 @@
         <v>7</v>
       </c>
       <c r="M1358" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="N1358" t="s">
         <v>77</v>
@@ -63858,7 +63858,7 @@
         <v>7</v>
       </c>
       <c r="M1359" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="N1359" t="s">
         <v>77</v>
@@ -64430,7 +64430,7 @@
         <v>7</v>
       </c>
       <c r="M1372" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="N1372" t="s">
         <v>77</v>
@@ -64694,7 +64694,7 @@
         <v>7</v>
       </c>
       <c r="M1378" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="N1378" t="s">
         <v>77</v>
@@ -64738,7 +64738,7 @@
         <v>7</v>
       </c>
       <c r="M1379" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="N1379" t="s">
         <v>77</v>
@@ -64782,7 +64782,7 @@
         <v>7</v>
       </c>
       <c r="M1380" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="N1380" t="s">
         <v>77</v>
@@ -65090,7 +65090,7 @@
         <v>7</v>
       </c>
       <c r="M1387" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="N1387" t="s">
         <v>77</v>
@@ -65134,7 +65134,7 @@
         <v>7</v>
       </c>
       <c r="M1388" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="N1388" t="s">
         <v>77</v>
@@ -65310,7 +65310,7 @@
         <v>7</v>
       </c>
       <c r="M1392" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="N1392" t="s">
         <v>77</v>
@@ -65706,7 +65706,7 @@
         <v>7</v>
       </c>
       <c r="M1401" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="N1401" t="s">
         <v>77</v>
@@ -65838,7 +65838,7 @@
         <v>7</v>
       </c>
       <c r="M1404" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="N1404" t="s">
         <v>77</v>
@@ -65882,7 +65882,7 @@
         <v>7</v>
       </c>
       <c r="M1405" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="N1405" t="s">
         <v>77</v>
@@ -66234,7 +66234,7 @@
         <v>7</v>
       </c>
       <c r="M1413" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="N1413" t="s">
         <v>77</v>
@@ -66278,7 +66278,7 @@
         <v>7</v>
       </c>
       <c r="M1414" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="N1414" t="s">
         <v>77</v>
@@ -66322,7 +66322,7 @@
         <v>7</v>
       </c>
       <c r="M1415" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="N1415" t="s">
         <v>77</v>
@@ -66454,7 +66454,7 @@
         <v>7</v>
       </c>
       <c r="M1418" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="N1418" t="s">
         <v>77</v>
@@ -66894,7 +66894,7 @@
         <v>7</v>
       </c>
       <c r="M1428" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="N1428" t="s">
         <v>77</v>
@@ -66982,7 +66982,7 @@
         <v>7</v>
       </c>
       <c r="M1430" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="N1430" t="s">
         <v>77</v>
@@ -67070,7 +67070,7 @@
         <v>7</v>
       </c>
       <c r="M1432" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="N1432" t="s">
         <v>77</v>
@@ -67774,7 +67774,7 @@
         <v>7</v>
       </c>
       <c r="M1448" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="N1448" t="s">
         <v>77</v>
@@ -69138,7 +69138,7 @@
         <v>7</v>
       </c>
       <c r="M1479" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="N1479" t="s">
         <v>77</v>
@@ -69358,7 +69358,7 @@
         <v>7</v>
       </c>
       <c r="M1484" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="N1484" t="s">
         <v>77</v>
@@ -69402,7 +69402,7 @@
         <v>7</v>
       </c>
       <c r="M1485" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="N1485" t="s">
         <v>77</v>
@@ -69490,7 +69490,7 @@
         <v>7</v>
       </c>
       <c r="M1487" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="N1487" t="s">
         <v>77</v>
@@ -69534,7 +69534,7 @@
         <v>7</v>
       </c>
       <c r="M1488" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="N1488" t="s">
         <v>77</v>
@@ -69578,7 +69578,7 @@
         <v>7</v>
       </c>
       <c r="M1489" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="N1489" t="s">
         <v>77</v>
@@ -69622,7 +69622,7 @@
         <v>7</v>
       </c>
       <c r="M1490" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="N1490" t="s">
         <v>77</v>
@@ -69886,7 +69886,7 @@
         <v>7</v>
       </c>
       <c r="M1496" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="N1496" t="s">
         <v>77</v>
@@ -70282,7 +70282,7 @@
         <v>7</v>
       </c>
       <c r="M1505" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="N1505" t="s">
         <v>77</v>
@@ -70414,7 +70414,7 @@
         <v>7</v>
       </c>
       <c r="M1508" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="N1508" t="s">
         <v>77</v>
@@ -70854,7 +70854,7 @@
         <v>7</v>
       </c>
       <c r="M1518" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="N1518" t="s">
         <v>77</v>
@@ -70898,7 +70898,7 @@
         <v>7</v>
       </c>
       <c r="M1519" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="N1519" t="s">
         <v>77</v>
@@ -71778,7 +71778,7 @@
         <v>7</v>
       </c>
       <c r="M1539" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="N1539" t="s">
         <v>77</v>
@@ -71822,7 +71822,7 @@
         <v>7</v>
       </c>
       <c r="M1540" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="N1540" t="s">
         <v>77</v>
@@ -71954,7 +71954,7 @@
         <v>7</v>
       </c>
       <c r="M1543" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="N1543" t="s">
         <v>77</v>
@@ -71998,7 +71998,7 @@
         <v>7</v>
       </c>
       <c r="M1544" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="N1544" t="s">
         <v>77</v>
@@ -72042,7 +72042,7 @@
         <v>7</v>
       </c>
       <c r="M1545" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="N1545" t="s">
         <v>77</v>
@@ -72086,7 +72086,7 @@
         <v>7</v>
       </c>
       <c r="M1546" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="N1546" t="s">
         <v>77</v>
@@ -72130,7 +72130,7 @@
         <v>7</v>
       </c>
       <c r="M1547" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="N1547" t="s">
         <v>77</v>
@@ -72262,7 +72262,7 @@
         <v>7</v>
       </c>
       <c r="M1550" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="N1550" t="s">
         <v>77</v>
@@ -72526,7 +72526,7 @@
         <v>7</v>
       </c>
       <c r="M1556" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="N1556" t="s">
         <v>77</v>
@@ -72570,7 +72570,7 @@
         <v>7</v>
       </c>
       <c r="M1557" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="N1557" t="s">
         <v>77</v>
@@ -73318,7 +73318,7 @@
         <v>7</v>
       </c>
       <c r="M1574" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="N1574" t="s">
         <v>77</v>
@@ -73406,7 +73406,7 @@
         <v>7</v>
       </c>
       <c r="M1576" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="N1576" t="s">
         <v>77</v>
@@ -73450,7 +73450,7 @@
         <v>7</v>
       </c>
       <c r="M1577" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="N1577" t="s">
         <v>77</v>
@@ -73494,7 +73494,7 @@
         <v>7</v>
       </c>
       <c r="M1578" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="N1578" t="s">
         <v>77</v>
@@ -74462,7 +74462,7 @@
         <v>7</v>
       </c>
       <c r="M1600" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="N1600" t="s">
         <v>77</v>
@@ -75166,7 +75166,7 @@
         <v>7</v>
       </c>
       <c r="M1616" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="N1616" t="s">
         <v>77</v>
@@ -75298,7 +75298,7 @@
         <v>7</v>
       </c>
       <c r="M1619" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="N1619" t="s">
         <v>77</v>
@@ -75342,7 +75342,7 @@
         <v>7</v>
       </c>
       <c r="M1620" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="N1620" t="s">
         <v>77</v>
@@ -75430,7 +75430,7 @@
         <v>7</v>
       </c>
       <c r="M1622" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="N1622" t="s">
         <v>77</v>
@@ -75738,7 +75738,7 @@
         <v>7</v>
       </c>
       <c r="M1629" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="N1629" t="s">
         <v>77</v>

</xml_diff>